<commit_message>
Upgrade NetSage AI to 50 cases + add Topology Explorer, Step-by-Step Pipeline View, and In-App Human Review Submission
</commit_message>
<xml_diff>
--- a/outputs/dashboard.xlsx
+++ b/outputs/dashboard.xlsx
@@ -223,12 +223,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$B$7:$B$14</f>
+              <f>'Dashboard'!$B$7:$B$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$C$7:$C$14</f>
+              <f>'Dashboard'!$C$7:$C$20</f>
             </numRef>
           </val>
         </ser>
@@ -382,7 +382,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!C17</f>
+              <f>'Dashboard'!C23</f>
             </strRef>
           </tx>
           <spPr>
@@ -392,12 +392,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$B$18:$B$20</f>
+              <f>'Dashboard'!$B$24:$B$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$C$18:$C$20</f>
+              <f>'Dashboard'!$C$24:$C$26</f>
             </numRef>
           </val>
         </ser>
@@ -812,7 +812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G24"/>
+  <dimension ref="B2:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B7)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B7)</f>
         <v/>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="G7" s="5">
-        <f>COUNTIF(Cases!$F$2:$F$31,F7)</f>
+        <f>COUNTIF(Cases!$F$2:$F$51,F7)</f>
         <v/>
       </c>
     </row>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B8)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B8)</f>
         <v/>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="G8" s="5">
-        <f>COUNTIF(Cases!$F$2:$F$31,F8)</f>
+        <f>COUNTIF(Cases!$F$2:$F$51,F8)</f>
         <v/>
       </c>
     </row>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B9)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B9)</f>
         <v/>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -928,18 +928,18 @@
         </is>
       </c>
       <c r="G9" s="5">
-        <f>COUNTIF(Cases!$F$2:$F$31,F9)</f>
+        <f>COUNTIF(Cases!$F$2:$F$51,F9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Gateway</t>
+          <t>EtherChannel</t>
         </is>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B10)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B10)</f>
         <v/>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -948,136 +948,202 @@
         </is>
       </c>
       <c r="G10" s="5">
-        <f>COUNTIF(Cases!$F$2:$F$31,F10)</f>
+        <f>COUNTIF(Cases!$F$2:$F$51,F10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>Gateway</t>
         </is>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B11)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Routing</t>
+          <t>HSRP</t>
         </is>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B12)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>VLAN</t>
+          <t>IPv6</t>
         </is>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B13)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Wireless</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIF(Cases!$B$2:$B$31,B14)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B14)</f>
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>QoS</t>
+        </is>
+      </c>
+      <c r="C15" s="5">
+        <f>COUNTIF(Cases!$B$2:$B$51,B15)</f>
+        <v/>
+      </c>
+    </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>AI vs Human Review Outcome</t>
-        </is>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Routing</t>
+        </is>
+      </c>
+      <c r="C16" s="5">
+        <f>COUNTIF(Cases!$B$2:$B$51,B16)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>STP</t>
+        </is>
+      </c>
+      <c r="C17" s="5">
+        <f>COUNTIF(Cases!$B$2:$B$51,B17)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIF(Review!$D$2:$D$31,B18)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Edited</t>
+          <t>VLAN</t>
         </is>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIF(Review!$D$2:$D$31,B19)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Wireless</t>
         </is>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIF(Review!$D$2:$D$31,B20)</f>
+        <f>COUNTIF(Cases!$B$2:$B$51,B20)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
+          <t>AI vs Human Review Outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="C24" s="5">
+        <f>COUNTIF(Review!$D$2:$D$51,B24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Edited</t>
+        </is>
+      </c>
+      <c r="C25" s="5">
+        <f>COUNTIF(Review!$D$2:$D$51,B25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="C26" s="5">
+        <f>COUNTIF(Review!$D$2:$D$51,B26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
           <t>Total cases:</t>
         </is>
       </c>
-      <c r="C22" s="5">
-        <f>COUNTA(Cases!$A$2:$A$31)</f>
+      <c r="C28" s="5">
+        <f>COUNTA(Cases!$A$2:$A$51)</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>AI agreement rate (Accepted / Total):</t>
         </is>
       </c>
-      <c r="C23" s="6">
-        <f>C18/SUM(C18:C20)</f>
+      <c r="C29" s="6">
+        <f>C24/SUM(C24:C26)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Cases needing correction (Edited + Rejected):</t>
         </is>
       </c>
-      <c r="C24" s="5">
-        <f>SUM(C19:C20)</f>
+      <c r="C30" s="5">
+        <f>SUM(C25:C26)</f>
         <v/>
       </c>
     </row>
@@ -1093,7 +1159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2096,6 +2162,646 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>C031</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>STP</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Network performance drops severely across the entire campus switch block due to massive frame flooding.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Core switch SW3 has default STP priority 32768, causing edge switch SW1 with a lower MAC address to win the Root election; suboptimal root placement causes excessive frame flooding across access uplinks.</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>C032</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>STP</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>An access port connected to an unmanaged hub repeatedly transitions between Forwarding and Blocking, causing packet loss.</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>BPDU Guard put Fa0/10 into err-disabled state after detecting rogue BPDUs from an unmanaged switch/hub plugged into a PortFast-enabled access port.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>C033</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>STP</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Hosts on VLAN 20 experience broadcast storms after a new redundant link was added between SW1 and SW2.</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>PortFast trunk was enabled on uplink Gi0/2, bypassing Listening and Learning states upon link up and causing an immediate temporary Layer 2 switching loop.</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>C034</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>EtherChannel</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>EtherChannel link between SW1 and SW2 shows Port-Channel 1 down, and individual member links are suspended.</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Speed mismatch on member interface Fa0/23 (SW1 is 100Mbps, SW2 is 10Mbps) prevents LACP bundling, causing member ports to be suspended.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>C035</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>EtherChannel</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Traffic distribution across a 4-link EtherChannel is heavily skewed; one link carries 90% of all traffic while others sit idle.</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>EtherChannel load-balancing hash is set to src-mac on a switch where all egress traffic originates from the same default gateway MAC, preventing traffic distribution across bundle links.</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>C036</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>HSRP</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Hosts on VLAN 10 use R1 as active gateway, but when R1's WAN link drops, traffic still routes to R1 instead of failing over to R2.</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>HSRP preempt is not enabled on R2. Even though R1's tracked WAN interface failed and reduced its priority to 90 (below R2's 100), R2 will not take over active status without preempt enabled.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>C037</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>HSRP</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Both R1 and R2 claim to be the Active HSRP gateway for VLAN 30, resulting in duplicate IP warnings and MAC address flapping on the switch.</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>HSRP hellos between R1 and R2 are blocked (or subinterfaces use mismatched HSRP authentication keys), leading both routers to believe the peer is dead and concurrently claim Active status.</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>C038</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>IPv6</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>IPv6-enabled workstations can ping local IPv6 link-local addresses but cannot reach external IPv6 global unicast destinations.</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Global 'ipv6 unicast-routing' is missing on router R1; without it, R1 acts only as an IPv6 end-host and will not forward IPv6 packets between interfaces or send Router Advertisements.</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>C039</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>IPv6</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Clients fail to acquire an IPv6 address automatically via SLAAC on VLAN 50.</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Router Advertisements are explicitly suppressed on G0/0.50 with 'ipv6 nd suppress-ra', preventing SLAAC clients from learning the network prefix and default gateway.</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>C040</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Connecting a new user desktop to switch port Fa0/12 immediately causes the port link LED to turn amber and shut down.</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Port security violation occurred on Fa0/12: incoming MAC address (00aa.bbcc.ddee) did not match the configured sticky MAC (0011.2233.4455), triggering the shutdown action.</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>C041</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Network administrator cannot SSH into R1 from the Management VLAN 40, getting 'Connection refused'.</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>VTY lines on R1 are configured with 'transport input telnet' instead of 'transport input ssh' (or 'all'), blocking encrypted SSH connection attempts on TCP port 22.</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Layer 7</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>C042</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Switch management access fails for all admin credentials when authentication server is unreachable.</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>AAA authentication is configured to use TACACS+ only without a 'local' fallback; when the TACACS+ server 10.40.1.5 is unreachable, admins are locked out.</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Layer 7</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>C043</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>QoS</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>VoIP phone calls experience severe jitter and audio clipping whenever large file downloads occur over the WAN link.</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>No QoS policy-map (LLQ / CBWFQ) is applied on WAN interface G0/1; default FIFO queuing drops latency-sensitive VoIP packets under link saturation.</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3/4</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>C044</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>QoS</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Differentiated Services Code Point (DSCP) EF markings set by IP phones are wiped out at the access switch.</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Access switch port Fa0/5 does not trust CoS/DSCP markings from the connected IP phone ('no mls qos trust'), overwriting incoming voice packets to DSCP 0 (Best Effort).</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2/3</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>C045</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>VLAN</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Inter-VLAN routing for VLAN 60 fails completely on router-on-a-stick topology while VLAN 10 and 20 work fine.</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Subinterface G0/0.60 has encapsulation mismatched to dot1Q 65 instead of dot1Q 60, causing tagged frames from VLAN 60 to be ignored by the subinterface.</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2/3</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>C046</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Routing</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>A router's CPU utilization spikes to 100% and traffic between two internal subnets is dropped due to TTL expired.</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Routing loop between R1 and R2 for destination network 172.20.0.0/16; both routers point to each other as the next-hop, causing packets to bounce until TTL expires.</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>C047</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>NAT</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Web server in DMZ (192.168.100.10) is unreachable from the internet on public IP 203.0.113.50.</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Static NAT rule maps public port 80 to internal port 808 instead of port 80 on the web server, causing external HTTP requests to hit a closed port.</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3/4</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>C048</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Admin host 10.40.1.100 cannot access web management on switch SW1, but pings succeed.</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Standard ACL 50 protecting the switch HTTP server permits 10.40.2.0/24 but omits admin subnet 10.40.1.0/24, denying web access while pinging (ICMP) remains unaffected.</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Layer 7</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>C049</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Routing</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>BGP session between R1 (AS 65001) and ISP router (AS 65002) stays in 'Active' or 'Idle' state indefinitely.</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>eBGP peer 198.51.100.1 is multiple hops away, but 'neighbor 198.51.100.1 ebgp-multihop' is not configured; default TTL of 1 drops eBGP packets before reaching the peer.</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Layer 3/4</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>C050</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>VLAN</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Laptops connected to IP Phone PC ports drop off the network whenever the phone reboots.</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Data VLAN and Voice VLAN on Fa0/9 are both set to VLAN 10. Voice and data must be on separate VLANs to allow proper 802.1Q tagging and prioritization.</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Layer 2</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2107,7 +2813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3110,6 +3816,646 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>C031</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Core switch SW3 has default STP priority 32768, causing edge switch SW1 with a lower MAC address to win the Root election; suboptimal root placement causes excessive frame flooding across access uplinks.</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Core switch SW3 has default STP priority 32768, causing edge switch SW1 with a lower MAC address to win the Root election; suboptimal root placement causes excessive frame flooding across access uplinks.</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>C032</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>BPDU Guard put Fa0/10 into err-disabled state after detecting rogue BPDUs from an unmanaged switch/hub plugged into a PortFast-enabled access port.</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>BPDU Guard put Fa0/10 into err-disabled state after detecting rogue BPDUs from an unmanaged switch/hub plugged into a PortFast-enabled access port.</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>C033</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>SW1 PortFast is globally disabled, causing temporary link blocking on trunk ports.</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>PortFast trunk was enabled on uplink Gi0/2, bypassing Listening and Learning states upon link up and causing an immediate temporary Layer 2 switching loop.</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>AI misdiagnosed PortFast trunk loop as missing global PortFast. Enabling PortFast globally would not stop the loop; the fix is to remove 'spanning-tree portfast trunk' from uplink Gi0/2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>C034</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Speed mismatch on member interface Fa0/23 (SW1 is 100Mbps, SW2 is 10Mbps) prevents LACP bundling, causing member ports to be suspended.</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Speed mismatch on member interface Fa0/23 (SW1 is 100Mbps, SW2 is 10Mbps) prevents LACP bundling, causing member ports to be suspended.</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>C035</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>EtherChannel load-balancing hash is set to src-mac on a switch where all egress traffic originates from the same default gateway MAC, preventing traffic distribution across bundle links.</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>EtherChannel load-balancing hash is set to src-mac on a switch where all egress traffic originates from the same default gateway MAC, preventing traffic distribution across bundle links.</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>C036</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>HSRP preempt is not enabled on R2. Even though R1's tracked WAN interface failed and reduced its priority to 90 (below R2's 100), R2 will not take over active status without preempt enabled.</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>HSRP preempt is not enabled on R2. Even though R1's tracked WAN interface failed and reduced its priority to 90 (below R2's 100), R2 will not take over active status without preempt enabled.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>C037</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>R1 and R2 have mismatched HSRP priority values causing active router contention.</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Edited</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>HSRP hellos between R1 and R2 are blocked (or subinterfaces use mismatched HSRP authentication keys), leading both routers to believe the peer is dead and concurrently claim Active status.</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>AI blamed HSRP priorities, but priority doesn't cause split-brain. The actual cause is blocked HSRP hellos or auth mismatch preventing peers from seeing each other. Corrected root_cause to hello/auth filtering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>C038</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Global 'ipv6 unicast-routing' is missing on router R1; without it, R1 acts only as an IPv6 end-host and will not forward IPv6 packets between interfaces or send Router Advertisements.</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Global 'ipv6 unicast-routing' is missing on router R1; without it, R1 acts only as an IPv6 end-host and will not forward IPv6 packets between interfaces or send Router Advertisements.</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>C039</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Router Advertisements are explicitly suppressed on G0/0.50 with 'ipv6 nd suppress-ra', preventing SLAAC clients from learning the network prefix and default gateway.</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Router Advertisements are explicitly suppressed on G0/0.50 with 'ipv6 nd suppress-ra', preventing SLAAC clients from learning the network prefix and default gateway.</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>C040</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Port security violation occurred on Fa0/12: incoming MAC address (00aa.bbcc.ddee) did not match the configured sticky MAC (0011.2233.4455), triggering the shutdown action.</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Port security violation occurred on Fa0/12: incoming MAC address (00aa.bbcc.ddee) did not match the configured sticky MAC (0011.2233.4455), triggering the shutdown action.</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>C041</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>VTY lines on R1 are configured with 'transport input telnet' instead of 'transport input ssh' (or 'all'), blocking encrypted SSH connection attempts on TCP port 22.</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>VTY lines on R1 are configured with 'transport input telnet' instead of 'transport input ssh' (or 'all'), blocking encrypted SSH connection attempts on TCP port 22.</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>C042</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>AAA authentication is configured to use TACACS+ only without a 'local' fallback; when the TACACS+ server 10.40.1.5 is unreachable, admins are locked out.</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>AAA authentication is configured to use TACACS+ only without a 'local' fallback; when the TACACS+ server 10.40.1.5 is unreachable, admins are locked out.</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>C043</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>No QoS policy-map (LLQ / CBWFQ) is applied on WAN interface G0/1; default FIFO queuing drops latency-sensitive VoIP packets under link saturation.</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>No QoS policy-map (LLQ / CBWFQ) is applied on WAN interface G0/1; default FIFO queuing drops latency-sensitive VoIP packets under link saturation.</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>C044</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Access switch port Fa0/5 does not trust CoS/DSCP markings from the connected IP phone ('no mls qos trust'), overwriting incoming voice packets to DSCP 0 (Best Effort).</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Access switch port Fa0/5 does not trust CoS/DSCP markings from the connected IP phone ('no mls qos trust'), overwriting incoming voice packets to DSCP 0 (Best Effort).</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>C045</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Subinterface G0/0.60 has encapsulation mismatched to dot1Q 65 instead of dot1Q 60, causing tagged frames from VLAN 60 to be ignored by the subinterface.</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Subinterface G0/0.60 has encapsulation mismatched to dot1Q 65 instead of dot1Q 60, causing tagged frames from VLAN 60 to be ignored by the subinterface.</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>C046</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Dest Subnet 172.20.0.0/16 is unroutable due to missing default gateway on R1.</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Routing loop between R1 and R2 for destination network 172.20.0.0/16; both routers point to each other as the next-hop, causing packets to bounce until TTL expires.</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>AI claimed default gateway was missing. The actual fault is a two-way static routing loop between R1 and R2 causing TTL expiration and CPU spikes. Corrected root_cause to routing loop removal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>C047</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Static NAT rule maps public port 80 to internal port 808 instead of port 80 on the web server, causing external HTTP requests to hit a closed port.</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Static NAT rule maps public port 80 to internal port 808 instead of port 80 on the web server, causing external HTTP requests to hit a closed port.</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>C048</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Standard ACL 50 protecting the switch HTTP server permits 10.40.2.0/24 but omits admin subnet 10.40.1.0/24, denying web access while pinging (ICMP) remains unaffected.</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Standard ACL 50 protecting the switch HTTP server permits 10.40.2.0/24 but omits admin subnet 10.40.1.0/24, denying web access while pinging (ICMP) remains unaffected.</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>C049</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>eBGP peer 198.51.100.1 is multiple hops away, but 'neighbor 198.51.100.1 ebgp-multihop' is not configured; default TTL of 1 drops eBGP packets before reaching the peer.</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>eBGP peer 198.51.100.1 is multiple hops away, but 'neighbor 198.51.100.1 ebgp-multihop' is not configured; default TTL of 1 drops eBGP packets before reaching the peer.</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>C050</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Data VLAN and Voice VLAN on Fa0/9 are both set to VLAN 10. Voice and data must be on separate VLANs to allow proper 802.1Q tagging and prioritization.</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Data VLAN and Voice VLAN on Fa0/9 are both set to VLAN 10. Voice and data must be on separate VLANs to allow proper 802.1Q tagging and prioritization.</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>AI diagnosis matched the evidence and known-correct root cause; approved as-is.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>